<commit_message>
Update item and ornament design docs
</commit_message>
<xml_diff>
--- a/spec/Docs/01_Design/CardDesignVersion/物品列表.xlsx
+++ b/spec/Docs/01_Design/CardDesignVersion/物品列表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\GodotProjects\Lost-Fragments\spec\Docs\01_Design\CardDesignVersion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E7B5BC-5747-4B36-AE78-D71897533EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4885F93-706F-48DF-8836-D6C87BAAC3FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="污染" sheetId="3" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="257">
   <si>
     <t>序号</t>
   </si>
@@ -223,18 +223,12 @@
     <t>废弃物/机械</t>
   </si>
   <si>
-    <t>梦境之种</t>
-  </si>
-  <si>
     <t>不可抽取</t>
   </si>
   <si>
     <t>4x4</t>
   </si>
   <si>
-    <t>5x5</t>
-  </si>
-  <si>
     <t>根源之梦</t>
   </si>
   <si>
@@ -486,6 +480,389 @@
   <si>
     <t>稀有道具</t>
     <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>梦境之种（1级形态）</t>
+  </si>
+  <si>
+    <t>等级1-9：被撞：+当前等级x1分。升级到10级时尝试变为2x2，若空间不足则掉出背包。</t>
+  </si>
+  <si>
+    <t>梦境之种的初始形态，用低占格提供稳定成长起点。</t>
+  </si>
+  <si>
+    <t>发光种子/小嫩芽</t>
+  </si>
+  <si>
+    <t>梦境之种（2级形态）</t>
+  </si>
+  <si>
+    <t>等级10-19：被撞：+当前等级x2分。升级到20级时尝试变为3x3，若空间不足则掉出背包。</t>
+  </si>
+  <si>
+    <t>第一次体型成长，开始要求玩家预留空间。</t>
+  </si>
+  <si>
+    <t>双叶幼苗/浅绿色梦光</t>
+  </si>
+  <si>
+    <t>梦境之种（3级形态）</t>
+  </si>
+  <si>
+    <t>等级20-29：被撞：+当前等级x4分。升级到30级时尝试变为4x4，若空间不足则掉出背包。</t>
+  </si>
+  <si>
+    <t>中后期核心收益形态，占格压力明显上升。</t>
+  </si>
+  <si>
+    <t>小型梦树/根须扩散</t>
+  </si>
+  <si>
+    <t>梦境之种（4级形态）</t>
+  </si>
+  <si>
+    <t>等级30及以上：被撞：+当前等级x8分。继续升级不会再次变大。</t>
+  </si>
+  <si>
+    <t>梦境流终端，巨大占格换取高额等级收益。</t>
+  </si>
+  <si>
+    <t>大型梦树/树冠发光</t>
+  </si>
+  <si>
+    <t>梦土铲</t>
+  </si>
+  <si>
+    <t>被撞：播种。</t>
+  </si>
+  <si>
+    <t>最基础的播种入口，让撞击链可以制造梦境之种。</t>
+  </si>
+  <si>
+    <t>沾着发光土壤的小铲</t>
+  </si>
+  <si>
+    <t>小喷壶</t>
+  </si>
+  <si>
+    <t>被撞：自身所指方向的第一个梦境之种等级+1；若没有命中梦境之种，+2分。</t>
+  </si>
+  <si>
+    <t>早期低成本升级工具，空场也不完全亏。</t>
+  </si>
+  <si>
+    <t>旧喷壶/蓝色水滴</t>
+  </si>
+  <si>
+    <t>空心果壳</t>
+  </si>
+  <si>
+    <t>从背包中丢弃时：在其原位置播种。若原位置已被占用，则在相邻空格播种。</t>
+  </si>
+  <si>
+    <t>把丢弃路线接入播种，并制造空间决策。</t>
+  </si>
+  <si>
+    <t>裂开的空果壳</t>
+  </si>
+  <si>
+    <t>种子铃铛</t>
+  </si>
+  <si>
+    <t>被撞：相邻所有梦境之种等级+1，每次结算最多影响2个。</t>
+  </si>
+  <si>
+    <t>鼓励把梦境之种围绕触发点摆放。</t>
+  </si>
+  <si>
+    <t>缠着幼芽的小铃铛</t>
+  </si>
+  <si>
+    <t>月露灯</t>
+  </si>
+  <si>
+    <t>每捕梦4次：随机1个梦境之种等级+1；若背包中没有梦境之种，则在随机空格播种。</t>
+  </si>
+  <si>
+    <t>提供稳定的梦种成长节奏，避免完全依赖撞击。</t>
+  </si>
+  <si>
+    <t>盛着月露的提灯</t>
+  </si>
+  <si>
+    <t>育苗托盘</t>
+  </si>
+  <si>
+    <t>每当你播种：+3分。每次捕梦后最多触发2次。</t>
+  </si>
+  <si>
+    <t>让前期多次播种有即时分数，不只服务后期。</t>
+  </si>
+  <si>
+    <t>旧木托盘/小苗格</t>
+  </si>
+  <si>
+    <t>根系导管</t>
+  </si>
+  <si>
+    <t>被撞：自身所指方向一整行中的所有梦境之种等级+1。</t>
+  </si>
+  <si>
+    <t>核心横向升级件，要求玩家规划方向和行列。</t>
+  </si>
+  <si>
+    <t>透明管道中流动的绿光</t>
+  </si>
+  <si>
+    <t>温室灯</t>
+  </si>
+  <si>
+    <t>每捕梦5次：等级最高的梦境之种等级+2。若因此变大，+12分。</t>
+  </si>
+  <si>
+    <t>稳定培养一个主种子，是纵向成长核心。</t>
+  </si>
+  <si>
+    <t>旧温室灯/暖色光圈</t>
+  </si>
+  <si>
+    <t>嫁接刀</t>
+  </si>
+  <si>
+    <t>被撞：相邻等级最低的梦境之种等级+2；若目标等级低于10，额外等级+1。</t>
+  </si>
+  <si>
+    <t>帮助新种子追赶等级，支持横向多种子。</t>
+  </si>
+  <si>
+    <t>银色小刀/藤蔓缠柄</t>
+  </si>
+  <si>
+    <t>蔓生罗盘</t>
+  </si>
+  <si>
+    <t>链结束：本次撞击链每命中1个梦境之种，使等级最高的梦境之种等级+1，最多+3。</t>
+  </si>
+  <si>
+    <t>把撞击链长度转化为梦种成长。</t>
+  </si>
+  <si>
+    <t>绿色罗盘/藤蔓指针</t>
+  </si>
+  <si>
+    <t>生态瓶</t>
+  </si>
+  <si>
+    <t>被撞：若背包中只有1个梦境之种，使其等级+3；否则所有梦境之种等级+1。</t>
+  </si>
+  <si>
+    <t>在单核巨树和多种子路线之间都能发挥作用。</t>
+  </si>
+  <si>
+    <t>玻璃生态瓶/瓶中小树</t>
+  </si>
+  <si>
+    <t>根网枢纽</t>
+  </si>
+  <si>
+    <t>被撞：每有1个相邻梦境之种，+5分，并使该梦境之种等级+1。</t>
+  </si>
+  <si>
+    <t>奖励密集摆放，是梦种与撞击站位的中期核心。</t>
+  </si>
+  <si>
+    <t>铜制根网节点</t>
+  </si>
+  <si>
+    <t>月冠温床</t>
+  </si>
+  <si>
+    <t>每个局内关卡第一次有梦境之种达到4x4：+60分。此后每捕梦4次，等级最高的梦境之种等级+2。</t>
+  </si>
+  <si>
+    <t>后期成型补强，奖励完成巨大梦种。</t>
+  </si>
+  <si>
+    <t>月冠形大型温床</t>
+  </si>
+  <si>
+    <t>星根祭坛</t>
+  </si>
+  <si>
+    <t>2x3</t>
+  </si>
+  <si>
+    <t>链结束：若本次撞击链命中过4x4梦境之种，+该梦境之种等级x3分。每个局内关卡限1次。</t>
+  </si>
+  <si>
+    <t>给4x4梦种一个高价值撞击终端。</t>
+  </si>
+  <si>
+    <t>星纹石祭坛/根须光路</t>
+  </si>
+  <si>
+    <t>巨木回声</t>
+  </si>
+  <si>
+    <t>每个局内关卡第一次4x4梦境之种被撞后：从该梦境之种发起一次撞击！</t>
+  </si>
+  <si>
+    <t>后期让巨大梦种从纯收益点变成撞击链节点。</t>
+  </si>
+  <si>
+    <t>树心回声纹/发光年轮</t>
+  </si>
+  <si>
+    <t>梦之种</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>机械/梦之种</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>铁珠</t>
+  </si>
+  <si>
+    <t>捕梦到另一枚铁珠时：撞击！</t>
+  </si>
+  <si>
+    <t>旧铁珠/轻微锈迹</t>
+  </si>
+  <si>
+    <t>小齿轮</t>
+  </si>
+  <si>
+    <t>被撞：+3分。若本次链已命中2个或以上机械物品，额外+2分。</t>
+  </si>
+  <si>
+    <t>小铜齿轮</t>
+  </si>
+  <si>
+    <t>传动皮带</t>
+  </si>
+  <si>
+    <t>被撞：+4分。若自身成功传导撞击，额外+3分。</t>
+  </si>
+  <si>
+    <t>黑色橡胶皮带</t>
+  </si>
+  <si>
+    <t>顺转弯管</t>
+  </si>
+  <si>
+    <t>机械/传动</t>
+  </si>
+  <si>
+    <t>被撞：顺转传动！每条链限1次。</t>
+  </si>
+  <si>
+    <t>L形铜管/顺时针标记</t>
+  </si>
+  <si>
+    <t>逆转弯管</t>
+  </si>
+  <si>
+    <t>被撞：逆转传动！每条链限1次。</t>
+  </si>
+  <si>
+    <t>L形铁管/逆时针标记</t>
+  </si>
+  <si>
+    <t>制动片</t>
+  </si>
+  <si>
+    <t>被撞：+8分，本条分支停止传导。</t>
+  </si>
+  <si>
+    <t>磨损刹车片</t>
+  </si>
+  <si>
+    <t>齿条</t>
+  </si>
+  <si>
+    <t>被撞：+本次链机械命中数分，最多+10分。若自身成功传导撞击，额外+4分。</t>
+  </si>
+  <si>
+    <t>长条齿轨</t>
+  </si>
+  <si>
+    <t>差速器</t>
+  </si>
+  <si>
+    <t>链结束：+本次链机械命中数x2分；若本次链转向次数大于等于2，额外+10分。</t>
+  </si>
+  <si>
+    <t>齿轮差速器</t>
+  </si>
+  <si>
+    <t>双轴转轮</t>
+  </si>
+  <si>
+    <t>被撞：若本次链机械命中数大于等于3，双向传动！每条链限1次。</t>
+  </si>
+  <si>
+    <t>双层转轮</t>
+  </si>
+  <si>
+    <t>蓄能飞轮</t>
+  </si>
+  <si>
+    <t>每当本次链累计命中3个机械物品：+12分。每条链最多触发2次。</t>
+  </si>
+  <si>
+    <t>发光飞轮</t>
+  </si>
+  <si>
+    <t>曲轴</t>
+  </si>
+  <si>
+    <t>被撞：逆转传动！若该传动命中机械物品，+10分。每条链限1次。</t>
+  </si>
+  <si>
+    <t>弯折曲轴</t>
+  </si>
+  <si>
+    <t>计数轮</t>
+  </si>
+  <si>
+    <t>链结束：若本次链命中大于等于6个物品，+18分；若大于等于9个，改为+32分。</t>
+  </si>
+  <si>
+    <t>数字计数轮</t>
+  </si>
+  <si>
+    <t>中央引擎</t>
+  </si>
+  <si>
+    <t>机械/核心</t>
+  </si>
+  <si>
+    <t>链结束：若本次链机械命中数大于等于10，+60分；若本次链转向次数大于等于3，额外+30分。</t>
+  </si>
+  <si>
+    <t>小型梦境引擎</t>
+  </si>
+  <si>
+    <t>终端计算机</t>
+  </si>
+  <si>
+    <t>链结束：+本次链机械命中数x3分，最多+45分；若本次链包含双向传动，额外+15分。</t>
+  </si>
+  <si>
+    <t>旧终端屏幕/齿轮接口</t>
+  </si>
+  <si>
+    <t>星环轴承</t>
+  </si>
+  <si>
+    <t>机械/传动/核心</t>
+  </si>
+  <si>
+    <t>每个局内关卡第一次被撞：全向传动！这些分支不能再次触发星环轴承。</t>
+  </si>
+  <si>
+    <t>星环形轴承</t>
   </si>
 </sst>
 </file>
@@ -677,8 +1054,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1062,7 +1439,7 @@
         <v>24</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>25</v>
@@ -1190,7 +1567,7 @@
         <v>24</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>38</v>
@@ -1302,7 +1679,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>48</v>
@@ -1339,7 +1716,7 @@
         <v>10</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>51</v>
@@ -1506,7 +1883,7 @@
         <v>24</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>60</v>
@@ -1543,7 +1920,7 @@
         <v>24</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>61</v>
@@ -1580,7 +1957,7 @@
         <v>24</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>60</v>
@@ -2081,36 +2458,474 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="8" max="8" width="76.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" t="s">
+        <v>210</v>
+      </c>
+      <c r="I2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>212</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" t="s">
+        <v>213</v>
+      </c>
+      <c r="I3" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>215</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4">
+        <v>8</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" t="s">
+        <v>216</v>
+      </c>
+      <c r="I4" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5" t="s">
+        <v>219</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
+        <v>220</v>
+      </c>
+      <c r="I5" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>222</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6" t="s">
+        <v>219</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>223</v>
+      </c>
+      <c r="I6" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>225</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
+        <v>226</v>
+      </c>
+      <c r="I7" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>228</v>
+      </c>
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+      <c r="G8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" t="s">
+        <v>229</v>
+      </c>
+      <c r="I8" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>231</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
+        <v>219</v>
+      </c>
+      <c r="F9">
+        <v>6</v>
+      </c>
+      <c r="G9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" t="s">
+        <v>232</v>
+      </c>
+      <c r="I9" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>234</v>
+      </c>
+      <c r="C10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10">
+        <v>18</v>
+      </c>
+      <c r="E10" t="s">
+        <v>219</v>
+      </c>
+      <c r="F10">
+        <v>8</v>
+      </c>
+      <c r="G10" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" t="s">
+        <v>235</v>
+      </c>
+      <c r="I10" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>237</v>
+      </c>
+      <c r="C11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11">
+        <v>18</v>
+      </c>
+      <c r="E11" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11">
+        <v>7</v>
+      </c>
+      <c r="G11" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" t="s">
+        <v>238</v>
+      </c>
+      <c r="I11" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>240</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>219</v>
+      </c>
+      <c r="F12">
+        <v>6</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" t="s">
+        <v>241</v>
+      </c>
+      <c r="I12" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>243</v>
+      </c>
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13">
+        <v>16</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13">
+        <v>6</v>
+      </c>
+      <c r="G13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" t="s">
+        <v>244</v>
+      </c>
+      <c r="I13" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>246</v>
+      </c>
+      <c r="C14" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14">
+        <v>28</v>
+      </c>
+      <c r="E14" t="s">
+        <v>247</v>
+      </c>
+      <c r="F14">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" t="s">
+        <v>248</v>
+      </c>
+      <c r="I14" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>250</v>
+      </c>
+      <c r="C15" t="s">
+        <v>199</v>
+      </c>
+      <c r="D15">
+        <v>30</v>
+      </c>
+      <c r="E15" t="s">
+        <v>247</v>
+      </c>
+      <c r="F15">
+        <v>16</v>
+      </c>
+      <c r="G15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" t="s">
+        <v>251</v>
+      </c>
+      <c r="I15" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>253</v>
+      </c>
+      <c r="C16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16">
+        <v>32</v>
+      </c>
+      <c r="E16" t="s">
+        <v>254</v>
+      </c>
+      <c r="F16">
+        <v>18</v>
+      </c>
+      <c r="G16" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" t="s">
+        <v>255</v>
+      </c>
+      <c r="I16" t="s">
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -2124,930 +2939,656 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="8" max="8" width="21" customWidth="1"/>
+    <col min="8" max="8" width="45.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="F2" t="s">
+        <v>207</v>
+      </c>
+      <c r="G2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" t="s">
+        <v>131</v>
+      </c>
+      <c r="I2" t="s">
+        <v>132</v>
+      </c>
+      <c r="J2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" t="s">
+        <v>207</v>
+      </c>
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" t="s">
+        <v>135</v>
+      </c>
+      <c r="I3" t="s">
+        <v>136</v>
+      </c>
+      <c r="J3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" t="s">
+        <v>207</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" t="s">
+        <v>139</v>
+      </c>
+      <c r="I4" t="s">
+        <v>140</v>
+      </c>
+      <c r="J4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" t="s">
+        <v>207</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" t="s">
+        <v>143</v>
+      </c>
+      <c r="I5" t="s">
+        <v>144</v>
+      </c>
+      <c r="J5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C6" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>207</v>
+      </c>
+      <c r="G6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" t="s">
+        <v>147</v>
+      </c>
+      <c r="I6" t="s">
+        <v>148</v>
+      </c>
+      <c r="J6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>150</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>207</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
+        <v>151</v>
+      </c>
+      <c r="I7" t="s">
+        <v>152</v>
+      </c>
+      <c r="J7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>207</v>
+      </c>
+      <c r="G8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H8" t="s">
+        <v>155</v>
+      </c>
+      <c r="I8" t="s">
+        <v>156</v>
+      </c>
+      <c r="J8" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9" t="s">
+        <v>207</v>
+      </c>
+      <c r="G9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" t="s">
+        <v>159</v>
+      </c>
+      <c r="I9" t="s">
+        <v>160</v>
+      </c>
+      <c r="J9" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>162</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10">
+        <v>8</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10" t="s">
+        <v>207</v>
+      </c>
+      <c r="G10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H10" t="s">
+        <v>163</v>
+      </c>
+      <c r="I10" t="s">
+        <v>164</v>
+      </c>
+      <c r="J10" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>166</v>
+      </c>
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11">
+        <v>8</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11" t="s">
+        <v>207</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>167</v>
+      </c>
+      <c r="I11" t="s">
+        <v>168</v>
+      </c>
+      <c r="J11" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>170</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12">
+        <v>12</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12" t="s">
+        <v>208</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" t="s">
+        <v>171</v>
+      </c>
+      <c r="I12" t="s">
+        <v>172</v>
+      </c>
+      <c r="J12" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>174</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13">
+        <v>15</v>
+      </c>
+      <c r="E13">
+        <v>6</v>
+      </c>
+      <c r="F13" t="s">
+        <v>208</v>
+      </c>
+      <c r="G13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" t="s">
+        <v>175</v>
+      </c>
+      <c r="I13" t="s">
+        <v>176</v>
+      </c>
+      <c r="J13" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14">
+        <v>12</v>
+      </c>
+      <c r="E14">
+        <v>5</v>
+      </c>
+      <c r="F14" t="s">
+        <v>207</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
+        <v>179</v>
+      </c>
+      <c r="I14" t="s">
+        <v>180</v>
+      </c>
+      <c r="J14" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15">
         <v>14</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G2" s="8" t="s">
+      <c r="B15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15">
+        <v>14</v>
+      </c>
+      <c r="E15">
+        <v>6</v>
+      </c>
+      <c r="F15" t="s">
+        <v>207</v>
+      </c>
+      <c r="G15" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-    </row>
-    <row r="3" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="8" t="s">
+      <c r="H15" t="s">
+        <v>183</v>
+      </c>
+      <c r="I15" t="s">
+        <v>184</v>
+      </c>
+      <c r="J15" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>186</v>
+      </c>
+      <c r="C16" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D16">
+        <v>18</v>
+      </c>
+      <c r="E16">
+        <v>7</v>
+      </c>
+      <c r="F16" t="s">
+        <v>207</v>
+      </c>
+      <c r="G16" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" t="s">
+        <v>187</v>
+      </c>
+      <c r="I16" t="s">
+        <v>188</v>
+      </c>
+      <c r="J16" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>190</v>
+      </c>
+      <c r="C17" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17">
+        <v>20</v>
+      </c>
+      <c r="E17">
+        <v>8</v>
+      </c>
+      <c r="F17" t="s">
+        <v>208</v>
+      </c>
+      <c r="G17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H17" t="s">
+        <v>191</v>
+      </c>
+      <c r="I17" t="s">
+        <v>192</v>
+      </c>
+      <c r="J17" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>194</v>
+      </c>
+      <c r="C18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18">
+        <v>25</v>
+      </c>
+      <c r="E18">
         <v>14</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G3" s="8" t="s">
+      <c r="F18" t="s">
+        <v>207</v>
+      </c>
+      <c r="G18" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-    </row>
-    <row r="4" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G4" s="8" t="s">
+      <c r="H18" t="s">
+        <v>195</v>
+      </c>
+      <c r="I18" t="s">
+        <v>196</v>
+      </c>
+      <c r="J18" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>198</v>
+      </c>
+      <c r="C19" t="s">
+        <v>199</v>
+      </c>
+      <c r="D19">
+        <v>30</v>
+      </c>
+      <c r="E19">
+        <v>16</v>
+      </c>
+      <c r="F19" t="s">
+        <v>207</v>
+      </c>
+      <c r="G19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" t="s">
+        <v>200</v>
+      </c>
+      <c r="I19" t="s">
+        <v>201</v>
+      </c>
+      <c r="J19" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>203</v>
+      </c>
+      <c r="C20" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20">
+        <v>26</v>
+      </c>
+      <c r="E20">
+        <v>15</v>
+      </c>
+      <c r="F20" t="s">
+        <v>207</v>
+      </c>
+      <c r="G20" t="s">
         <v>24</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-    </row>
-    <row r="5" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-    </row>
-    <row r="6" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-    </row>
-    <row r="7" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-    </row>
-    <row r="8" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-    </row>
-    <row r="9" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-    </row>
-    <row r="10" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-    </row>
-    <row r="11" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-    </row>
-    <row r="12" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-    </row>
-    <row r="13" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-    </row>
-    <row r="14" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-    </row>
-    <row r="15" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-    </row>
-    <row r="16" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-    </row>
-    <row r="17" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-    </row>
-    <row r="18" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-    </row>
-    <row r="19" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-    </row>
-    <row r="20" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-    </row>
-    <row r="21" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-    </row>
-    <row r="22" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-    </row>
-    <row r="23" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-    </row>
-    <row r="24" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-    </row>
-    <row r="25" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-    </row>
-    <row r="26" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
-    </row>
-    <row r="27" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
-    </row>
-    <row r="28" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
-    </row>
-    <row r="29" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="8"/>
-    </row>
-    <row r="30" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
-    </row>
-    <row r="31" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A31" s="8"/>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
-      <c r="J31" s="8"/>
-    </row>
-    <row r="32" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A32" s="8"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
-      <c r="J32" s="8"/>
-    </row>
-    <row r="33" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A33" s="8"/>
-      <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
-      <c r="J33" s="8"/>
-    </row>
-    <row r="34" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A34" s="8"/>
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="8"/>
-    </row>
-    <row r="35" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A35" s="8"/>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-    </row>
-    <row r="36" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A36" s="8"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="8"/>
-    </row>
-    <row r="37" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A37" s="8"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8"/>
-      <c r="I37" s="8"/>
-      <c r="J37" s="8"/>
-    </row>
-    <row r="38" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A38" s="8"/>
-      <c r="B38" s="8"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
-      <c r="J38" s="8"/>
-    </row>
-    <row r="39" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A39" s="8"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="8"/>
-    </row>
-    <row r="40" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A40" s="8"/>
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="8"/>
-    </row>
-    <row r="41" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A41" s="8"/>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="8"/>
-      <c r="I41" s="8"/>
-      <c r="J41" s="8"/>
-    </row>
-    <row r="42" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A42" s="8"/>
-      <c r="B42" s="8"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
-      <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="8"/>
-      <c r="I42" s="8"/>
-      <c r="J42" s="8"/>
-    </row>
-    <row r="43" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A43" s="8"/>
-      <c r="B43" s="8"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
-      <c r="E43" s="8"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="8"/>
-      <c r="I43" s="8"/>
-      <c r="J43" s="8"/>
-    </row>
-    <row r="44" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A44" s="8"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
-      <c r="G44" s="8"/>
-      <c r="H44" s="8"/>
-      <c r="I44" s="8"/>
-      <c r="J44" s="8"/>
-    </row>
-    <row r="45" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A45" s="8"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="8"/>
-      <c r="I45" s="8"/>
-      <c r="J45" s="8"/>
-    </row>
-    <row r="46" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A46" s="8"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="8"/>
-      <c r="F46" s="8"/>
-      <c r="G46" s="8"/>
-      <c r="H46" s="8"/>
-      <c r="I46" s="8"/>
-      <c r="J46" s="8"/>
-    </row>
-    <row r="47" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A47" s="8"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
-      <c r="I47" s="8"/>
-      <c r="J47" s="8"/>
-    </row>
-    <row r="48" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A48" s="8"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
-      <c r="F48" s="8"/>
-      <c r="G48" s="8"/>
-      <c r="H48" s="8"/>
-      <c r="I48" s="8"/>
-      <c r="J48" s="8"/>
-    </row>
-    <row r="49" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A49" s="8"/>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="8"/>
-      <c r="I49" s="8"/>
-      <c r="J49" s="8"/>
-    </row>
-    <row r="50" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A50" s="8"/>
-      <c r="B50" s="8"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="8"/>
-      <c r="F50" s="8"/>
-      <c r="G50" s="8"/>
-      <c r="H50" s="8"/>
-      <c r="I50" s="8"/>
-      <c r="J50" s="8"/>
-    </row>
-    <row r="51" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A51" s="8"/>
-      <c r="B51" s="8"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="8"/>
-      <c r="G51" s="8"/>
-      <c r="H51" s="8"/>
-      <c r="I51" s="8"/>
-      <c r="J51" s="8"/>
-    </row>
-    <row r="52" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A52" s="8"/>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="8"/>
-      <c r="E52" s="8"/>
-      <c r="F52" s="8"/>
-      <c r="G52" s="8"/>
-      <c r="H52" s="8"/>
-      <c r="I52" s="8"/>
-      <c r="J52" s="8"/>
-    </row>
-    <row r="53" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A53" s="8"/>
-      <c r="B53" s="8"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="8"/>
-      <c r="F53" s="8"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="8"/>
-      <c r="I53" s="8"/>
-      <c r="J53" s="8"/>
-    </row>
-    <row r="54" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A54" s="8"/>
-      <c r="B54" s="8"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="8"/>
-      <c r="E54" s="8"/>
-      <c r="F54" s="8"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="8"/>
-      <c r="I54" s="8"/>
-      <c r="J54" s="8"/>
-    </row>
-    <row r="55" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A55" s="8"/>
-      <c r="B55" s="8"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="8"/>
-      <c r="E55" s="8"/>
-      <c r="F55" s="8"/>
-      <c r="G55" s="8"/>
-      <c r="H55" s="8"/>
-      <c r="I55" s="8"/>
-      <c r="J55" s="8"/>
-    </row>
-    <row r="56" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A56" s="8"/>
-      <c r="B56" s="8"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="8"/>
-      <c r="E56" s="8"/>
-      <c r="F56" s="8"/>
-      <c r="G56" s="8"/>
-      <c r="H56" s="8"/>
-      <c r="I56" s="8"/>
-      <c r="J56" s="8"/>
-    </row>
-    <row r="57" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A57" s="8"/>
-      <c r="B57" s="8"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="8"/>
-      <c r="E57" s="8"/>
-      <c r="F57" s="8"/>
-      <c r="G57" s="8"/>
-      <c r="H57" s="8"/>
-      <c r="I57" s="8"/>
-      <c r="J57" s="8"/>
-    </row>
-    <row r="58" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A58" s="8"/>
-      <c r="B58" s="8"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="8"/>
-      <c r="E58" s="8"/>
-      <c r="F58" s="8"/>
-      <c r="G58" s="8"/>
-      <c r="H58" s="8"/>
-      <c r="I58" s="8"/>
-      <c r="J58" s="8"/>
-    </row>
-    <row r="59" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A59" s="8"/>
-      <c r="B59" s="8"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="8"/>
-      <c r="E59" s="8"/>
-      <c r="F59" s="8"/>
-      <c r="G59" s="8"/>
-      <c r="H59" s="8"/>
-      <c r="I59" s="8"/>
-      <c r="J59" s="8"/>
-    </row>
-    <row r="60" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A60" s="8"/>
-      <c r="B60" s="8"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="8"/>
-      <c r="E60" s="8"/>
-      <c r="F60" s="8"/>
-      <c r="G60" s="8"/>
-      <c r="H60" s="8"/>
-      <c r="I60" s="8"/>
-      <c r="J60" s="8"/>
-    </row>
-    <row r="61" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A61" s="8"/>
-      <c r="B61" s="8"/>
-      <c r="C61" s="8"/>
-      <c r="D61" s="8"/>
-      <c r="E61" s="8"/>
-      <c r="F61" s="8"/>
-      <c r="G61" s="8"/>
-      <c r="H61" s="8"/>
-      <c r="I61" s="8"/>
-      <c r="J61" s="8"/>
-    </row>
-    <row r="62" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A62" s="8"/>
-      <c r="B62" s="8"/>
-      <c r="C62" s="8"/>
-      <c r="D62" s="8"/>
-      <c r="E62" s="8"/>
-      <c r="F62" s="8"/>
-      <c r="G62" s="8"/>
-      <c r="H62" s="8"/>
-      <c r="I62" s="8"/>
-      <c r="J62" s="8"/>
-    </row>
-    <row r="63" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A63" s="8"/>
-      <c r="B63" s="8"/>
-      <c r="C63" s="8"/>
-      <c r="D63" s="8"/>
-      <c r="E63" s="8"/>
-      <c r="F63" s="8"/>
-      <c r="G63" s="8"/>
-      <c r="H63" s="8"/>
-      <c r="I63" s="8"/>
-      <c r="J63" s="8"/>
-    </row>
-    <row r="64" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A64" s="8"/>
-      <c r="B64" s="8"/>
-      <c r="C64" s="8"/>
-      <c r="D64" s="8"/>
-      <c r="E64" s="8"/>
-      <c r="F64" s="8"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="8"/>
-      <c r="I64" s="8"/>
-      <c r="J64" s="8"/>
-    </row>
-    <row r="65" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A65" s="8"/>
-      <c r="B65" s="8"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="8"/>
-      <c r="E65" s="8"/>
-      <c r="F65" s="8"/>
-      <c r="G65" s="8"/>
-      <c r="H65" s="8"/>
-      <c r="I65" s="8"/>
-      <c r="J65" s="8"/>
-    </row>
-    <row r="66" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A66" s="8"/>
-      <c r="B66" s="8"/>
-      <c r="C66" s="8"/>
-      <c r="D66" s="8"/>
-      <c r="E66" s="8"/>
-      <c r="F66" s="8"/>
-      <c r="G66" s="8"/>
-      <c r="H66" s="8"/>
-      <c r="I66" s="8"/>
-      <c r="J66" s="8"/>
-    </row>
-    <row r="67" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A67" s="8"/>
-      <c r="B67" s="8"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="8"/>
-      <c r="E67" s="8"/>
-      <c r="F67" s="8"/>
-      <c r="G67" s="8"/>
-      <c r="H67" s="8"/>
-      <c r="I67" s="8"/>
-      <c r="J67" s="8"/>
-    </row>
-    <row r="68" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A68" s="8"/>
-      <c r="B68" s="8"/>
-      <c r="C68" s="8"/>
-      <c r="D68" s="8"/>
-      <c r="E68" s="8"/>
-      <c r="F68" s="8"/>
-      <c r="G68" s="8"/>
-      <c r="H68" s="8"/>
-      <c r="I68" s="8"/>
-      <c r="J68" s="8"/>
-    </row>
-    <row r="69" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A69" s="8"/>
-      <c r="B69" s="8"/>
-      <c r="C69" s="8"/>
-      <c r="D69" s="8"/>
-      <c r="E69" s="8"/>
-      <c r="F69" s="8"/>
-      <c r="G69" s="8"/>
-      <c r="H69" s="8"/>
-      <c r="I69" s="8"/>
-      <c r="J69" s="8"/>
-    </row>
-    <row r="70" spans="1:10" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A70" s="8"/>
-      <c r="B70" s="8"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="8"/>
-      <c r="E70" s="8"/>
-      <c r="F70" s="8"/>
-      <c r="G70" s="8"/>
-      <c r="H70" s="8"/>
-      <c r="I70" s="8"/>
-      <c r="J70" s="8"/>
+      <c r="H20" t="s">
+        <v>204</v>
+      </c>
+      <c r="I20" t="s">
+        <v>205</v>
+      </c>
+      <c r="J20" t="s">
+        <v>206</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="B2:B6"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B2:B5"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3099,25 +3640,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -3125,10 +3666,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D3">
         <v>5</v>
@@ -3137,7 +3678,7 @@
         <v>1</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>9</v>
@@ -3148,10 +3689,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D4">
         <v>5</v>
@@ -3160,10 +3701,10 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -3171,10 +3712,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D5">
         <v>12</v>
@@ -3183,10 +3724,10 @@
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -3194,10 +3735,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D6">
         <v>8</v>
@@ -3206,10 +3747,10 @@
         <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -3217,10 +3758,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D7">
         <v>10</v>
@@ -3229,10 +3770,10 @@
         <v>3</v>
       </c>
       <c r="G7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H7" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -3240,10 +3781,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D8">
         <v>5</v>
@@ -3252,10 +3793,10 @@
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -3263,25 +3804,25 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D9">
         <v>2</v>
       </c>
       <c r="E9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -3289,10 +3830,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D10">
         <v>10</v>
@@ -3301,10 +3842,10 @@
         <v>4</v>
       </c>
       <c r="G10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -3312,10 +3853,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D11">
         <v>10</v>
@@ -3324,10 +3865,10 @@
         <v>4</v>
       </c>
       <c r="G11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -3335,10 +3876,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D12">
         <v>20</v>
@@ -3347,13 +3888,13 @@
         <v>15</v>
       </c>
       <c r="F12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -3604,10 +4145,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D2">
         <v>5</v>
@@ -3616,13 +4157,13 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G2" t="s">
         <v>106</v>
       </c>
-      <c r="G2" t="s">
-        <v>108</v>
-      </c>
       <c r="H2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -3630,10 +4171,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D3">
         <v>5</v>
@@ -3642,13 +4183,13 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
+        <v>104</v>
+      </c>
+      <c r="G3" t="s">
         <v>106</v>
       </c>
-      <c r="G3" t="s">
-        <v>108</v>
-      </c>
       <c r="H3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -3656,7 +4197,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
@@ -3668,13 +4209,13 @@
         <v>2</v>
       </c>
       <c r="F4" t="s">
+        <v>104</v>
+      </c>
+      <c r="G4" t="s">
         <v>106</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>108</v>
-      </c>
-      <c r="H4" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -3682,7 +4223,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C5" t="s">
         <v>23</v>
@@ -3694,13 +4235,13 @@
         <v>2</v>
       </c>
       <c r="F5" t="s">
+        <v>104</v>
+      </c>
+      <c r="G5" t="s">
         <v>106</v>
       </c>
-      <c r="G5" t="s">
-        <v>108</v>
-      </c>
       <c r="H5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -3708,7 +4249,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C6" t="s">
         <v>23</v>
@@ -3720,13 +4261,13 @@
         <v>2</v>
       </c>
       <c r="F6" t="s">
+        <v>104</v>
+      </c>
+      <c r="G6" t="s">
         <v>106</v>
       </c>
-      <c r="G6" t="s">
-        <v>108</v>
-      </c>
       <c r="H6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -3734,7 +4275,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C7" t="s">
         <v>23</v>
@@ -3746,13 +4287,13 @@
         <v>3</v>
       </c>
       <c r="F7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G7" t="s">
         <v>106</v>
       </c>
-      <c r="G7" t="s">
-        <v>108</v>
-      </c>
       <c r="H7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -3760,7 +4301,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C8" t="s">
         <v>23</v>
@@ -3772,13 +4313,13 @@
         <v>3</v>
       </c>
       <c r="F8" t="s">
+        <v>104</v>
+      </c>
+      <c r="G8" t="s">
         <v>106</v>
       </c>
-      <c r="G8" t="s">
-        <v>108</v>
-      </c>
       <c r="H8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -3786,7 +4327,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C9" t="s">
         <v>23</v>
@@ -3798,13 +4339,13 @@
         <v>2</v>
       </c>
       <c r="F9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G9" t="s">
         <v>106</v>
       </c>
-      <c r="G9" t="s">
-        <v>108</v>
-      </c>
       <c r="H9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -3812,7 +4353,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
@@ -3824,13 +4365,13 @@
         <v>3</v>
       </c>
       <c r="F10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G10" t="s">
         <v>106</v>
       </c>
-      <c r="G10" t="s">
-        <v>108</v>
-      </c>
       <c r="H10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -3838,10 +4379,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D11">
         <v>18</v>
@@ -3850,13 +4391,13 @@
         <v>3</v>
       </c>
       <c r="F11" t="s">
+        <v>104</v>
+      </c>
+      <c r="G11" t="s">
         <v>106</v>
       </c>
-      <c r="G11" t="s">
-        <v>108</v>
-      </c>
       <c r="H11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -3867,10 +4408,10 @@
         <v>23</v>
       </c>
       <c r="F12" t="s">
+        <v>104</v>
+      </c>
+      <c r="G12" t="s">
         <v>106</v>
-      </c>
-      <c r="G12" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -3881,10 +4422,10 @@
         <v>23</v>
       </c>
       <c r="F13" t="s">
+        <v>104</v>
+      </c>
+      <c r="G13" t="s">
         <v>106</v>
-      </c>
-      <c r="G13" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -3895,10 +4436,10 @@
         <v>23</v>
       </c>
       <c r="F14" t="s">
+        <v>104</v>
+      </c>
+      <c r="G14" t="s">
         <v>106</v>
-      </c>
-      <c r="G14" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -3909,10 +4450,10 @@
         <v>23</v>
       </c>
       <c r="F15" t="s">
+        <v>104</v>
+      </c>
+      <c r="G15" t="s">
         <v>106</v>
-      </c>
-      <c r="G15" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -3923,10 +4464,10 @@
         <v>23</v>
       </c>
       <c r="F16" t="s">
+        <v>104</v>
+      </c>
+      <c r="G16" t="s">
         <v>106</v>
-      </c>
-      <c r="G16" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -3937,10 +4478,10 @@
         <v>23</v>
       </c>
       <c r="F17" t="s">
+        <v>104</v>
+      </c>
+      <c r="G17" t="s">
         <v>106</v>
-      </c>
-      <c r="G17" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -3951,10 +4492,10 @@
         <v>23</v>
       </c>
       <c r="F18" t="s">
+        <v>104</v>
+      </c>
+      <c r="G18" t="s">
         <v>106</v>
-      </c>
-      <c r="G18" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -3965,10 +4506,10 @@
         <v>23</v>
       </c>
       <c r="F19" t="s">
+        <v>104</v>
+      </c>
+      <c r="G19" t="s">
         <v>106</v>
-      </c>
-      <c r="G19" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
@@ -3979,10 +4520,10 @@
         <v>23</v>
       </c>
       <c r="F20" t="s">
+        <v>104</v>
+      </c>
+      <c r="G20" t="s">
         <v>106</v>
-      </c>
-      <c r="G20" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
@@ -3990,7 +4531,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C21" t="s">
         <v>23</v>
@@ -4002,13 +4543,13 @@
         <v>7</v>
       </c>
       <c r="F21" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G21" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H21" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -4019,10 +4560,10 @@
         <v>23</v>
       </c>
       <c r="F22" t="s">
+        <v>104</v>
+      </c>
+      <c r="G22" t="s">
         <v>106</v>
-      </c>
-      <c r="G22" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
@@ -4033,10 +4574,10 @@
         <v>23</v>
       </c>
       <c r="F23" t="s">
+        <v>104</v>
+      </c>
+      <c r="G23" t="s">
         <v>106</v>
-      </c>
-      <c r="G23" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
@@ -4047,10 +4588,10 @@
         <v>23</v>
       </c>
       <c r="F24" t="s">
+        <v>104</v>
+      </c>
+      <c r="G24" t="s">
         <v>106</v>
-      </c>
-      <c r="G24" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
@@ -4061,10 +4602,10 @@
         <v>23</v>
       </c>
       <c r="F25" t="s">
+        <v>104</v>
+      </c>
+      <c r="G25" t="s">
         <v>106</v>
-      </c>
-      <c r="G25" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
@@ -4075,10 +4616,10 @@
         <v>23</v>
       </c>
       <c r="F26" t="s">
+        <v>104</v>
+      </c>
+      <c r="G26" t="s">
         <v>106</v>
-      </c>
-      <c r="G26" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
@@ -4089,10 +4630,10 @@
         <v>23</v>
       </c>
       <c r="F27" t="s">
+        <v>104</v>
+      </c>
+      <c r="G27" t="s">
         <v>106</v>
-      </c>
-      <c r="G27" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
@@ -4103,10 +4644,10 @@
         <v>23</v>
       </c>
       <c r="F28" t="s">
+        <v>104</v>
+      </c>
+      <c r="G28" t="s">
         <v>106</v>
-      </c>
-      <c r="G28" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
@@ -4117,10 +4658,10 @@
         <v>23</v>
       </c>
       <c r="F29" t="s">
+        <v>104</v>
+      </c>
+      <c r="G29" t="s">
         <v>106</v>
-      </c>
-      <c r="G29" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
@@ -4131,10 +4672,10 @@
         <v>23</v>
       </c>
       <c r="F30" t="s">
+        <v>104</v>
+      </c>
+      <c r="G30" t="s">
         <v>106</v>
-      </c>
-      <c r="G30" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
@@ -4145,10 +4686,10 @@
         <v>23</v>
       </c>
       <c r="F31" t="s">
+        <v>104</v>
+      </c>
+      <c r="G31" t="s">
         <v>106</v>
-      </c>
-      <c r="G31" t="s">
-        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove pollution backlash and replace isolation box
</commit_message>
<xml_diff>
--- a/spec/Docs/01_Design/CardDesignVersion/物品列表.xlsx
+++ b/spec/Docs/01_Design/CardDesignVersion/物品列表.xlsx
@@ -1,34 +1,44 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\GodotProjects\Lost-Fragments\spec\Docs\01_Design\CardDesignVersion\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4885F93-706F-48DF-8836-D6C87BAAC3FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="污染" sheetId="3" r:id="rId1"/>
-    <sheet name="机械" sheetId="4" r:id="rId2"/>
-    <sheet name="梦境之种" sheetId="5" r:id="rId3"/>
-    <sheet name="通用" sheetId="6" r:id="rId4"/>
-    <sheet name="道具" sheetId="7" r:id="rId5"/>
-  </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <TotalTime>0</TotalTime>
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>工作表</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>5</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="5" baseType="lpstr">
+      <vt:lpstr>污染</vt:lpstr>
+      <vt:lpstr>机械</vt:lpstr>
+      <vt:lpstr>梦境之种</vt:lpstr>
+      <vt:lpstr>通用</vt:lpstr>
+      <vt:lpstr>道具</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <cp:lastModifiedBy>Isaccson August</cp:lastModifiedBy>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-05-14T06:48:51Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="232">
   <si>
     <t>序号</t>
@@ -184,15 +194,11 @@
   <si>
     <t>被撞：相邻所有废弃物+1污染</t>
   </si>
-  <si>
-    <t>隔离箱</t>
-  </si>
+  <si>污封箱</si>
   <si>
     <t>机械</t>
   </si>
-  <si>
-    <t>污染层数导致的梦值扣除效应-1</t>
-  </si>
+  <si>被撞：所指方向第一个物品污染+1；若目标已有污染，则本次撞击结算结束后相邻1格内随机1个物品污染+1。</si>
   <si>
     <t>旧足球</t>
   </si>
@@ -767,7 +773,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -974,7 +980,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1269,7 +1275,36 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\GodotProjects\Lost-Fragments\spec\Docs\01_Design\CardDesignVersion\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4885F93-706F-48DF-8836-D6C87BAAC3FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
+  <sheets>
+    <sheet name="污染" sheetId="3" r:id="rId1"/>
+    <sheet name="机械" sheetId="4" r:id="rId2"/>
+    <sheet name="梦境之种" sheetId="5" r:id="rId3"/>
+    <sheet name="通用" sheetId="6" r:id="rId4"/>
+    <sheet name="道具" sheetId="7" r:id="rId5"/>
+  </sheets>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DB9B9BD-AF62-4C4D-AEE8-E856B9FC7F56}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2353,7 +2388,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr" xr:uid="{46BC56F0-F526-4B1D-8544-516A0AD02E1A}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2834,7 +2869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr" xr:uid="{DD51D4CC-8D74-4158-BD3D-2E74B32B1C81}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3495,7 +3530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8133C797-C29D-4E8F-AE0A-941547D59A04}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3997,7 +4032,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr">
   <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>